<commit_message>
2026-09-05 changes - airflow changes - workflow mechanism, pass training notebook in config - additional attributes in pre-process (6m to 3y ratios)
</commit_message>
<xml_diff>
--- a/src/Model-Training/LightGBM_v3/selected_features.xlsx
+++ b/src/Model-Training/LightGBM_v3/selected_features.xlsx
@@ -8,19 +8,22 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="A:\Dominic\My Projects\Home Credit\src\Model-Training\LightGBM_v3\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{115E215D-6348-48BB-99FD-B85E8B3C307F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{18B59CCB-5B4B-4B28-B978-69906345919B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="2616" yWindow="2616" windowWidth="17280" windowHeight="8880" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="228" windowWidth="23040" windowHeight="12012" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="0"/>
+  <definedNames>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Sheet1!$A$1:$A$26</definedName>
+  </definedNames>
+  <calcPr calcId="191029"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="27" uniqueCount="27">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="26" uniqueCount="26">
   <si>
     <t>feature</t>
   </si>
@@ -62,9 +65,6 @@
   </si>
   <si>
     <t>BUREAUCREDIT_DAYS_CREDIT_UPDATE_MEAN</t>
-  </si>
-  <si>
-    <t>DAYS_EMPLOYED</t>
   </si>
   <si>
     <t>DAYS_ID_PUBLISH</t>
@@ -464,7 +464,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:A27"/>
+  <dimension ref="A1:A26"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="60.77734375" bestFit="1" customWidth="1"/>
@@ -477,107 +477,107 @@
     </row>
     <row r="2" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
-        <v>1</v>
+        <v>16</v>
       </c>
     </row>
     <row r="3" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
-        <v>2</v>
+        <v>5</v>
       </c>
     </row>
     <row r="4" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
-        <v>3</v>
+        <v>6</v>
       </c>
     </row>
     <row r="5" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
-        <v>4</v>
+        <v>13</v>
       </c>
     </row>
     <row r="6" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
-        <v>5</v>
+        <v>17</v>
       </c>
     </row>
     <row r="7" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
-        <v>6</v>
+        <v>21</v>
       </c>
     </row>
     <row r="8" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
     </row>
     <row r="9" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A9" t="s">
-        <v>8</v>
+        <v>14</v>
       </c>
     </row>
     <row r="10" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A10" t="s">
-        <v>9</v>
+        <v>19</v>
       </c>
     </row>
     <row r="11" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A11" t="s">
-        <v>10</v>
+        <v>20</v>
       </c>
     </row>
     <row r="12" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A12" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
     </row>
     <row r="13" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A13" t="s">
-        <v>12</v>
+        <v>4</v>
       </c>
     </row>
     <row r="14" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A14" t="s">
-        <v>13</v>
+        <v>25</v>
       </c>
     </row>
     <row r="15" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A15" t="s">
-        <v>14</v>
+        <v>9</v>
       </c>
     </row>
     <row r="16" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A16" t="s">
-        <v>15</v>
+        <v>10</v>
       </c>
     </row>
     <row r="17" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A17" t="s">
-        <v>16</v>
+        <v>1</v>
       </c>
     </row>
     <row r="18" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A18" t="s">
-        <v>17</v>
+        <v>15</v>
       </c>
     </row>
     <row r="19" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A19" t="s">
-        <v>18</v>
+        <v>3</v>
       </c>
     </row>
     <row r="20" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A20" t="s">
-        <v>19</v>
+        <v>7</v>
       </c>
     </row>
     <row r="21" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A21" t="s">
-        <v>20</v>
+        <v>11</v>
       </c>
     </row>
     <row r="22" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A22" t="s">
-        <v>21</v>
+        <v>24</v>
       </c>
     </row>
     <row r="23" spans="1:1" x14ac:dyDescent="0.3">
@@ -592,20 +592,21 @@
     </row>
     <row r="25" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A25" t="s">
-        <v>24</v>
+        <v>2</v>
       </c>
     </row>
     <row r="26" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A26" t="s">
-        <v>25</v>
-      </c>
-    </row>
-    <row r="27" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A27" t="s">
-        <v>26</v>
+        <v>18</v>
       </c>
     </row>
   </sheetData>
+  <autoFilter ref="A1:A26" xr:uid="{00000000-0001-0000-0000-000000000000}">
+    <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:A26">
+      <sortCondition ref="A1:A26"/>
+    </sortState>
+  </autoFilter>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <pageSetup orientation="portrait" r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>